<commit_message>
docs: replace raw HTTP status codes in Black Box sheets with realistic business outcomes and error reasons
</commit_message>
<xml_diff>
--- a/test/PBL_Black_Box_Testing.xlsx
+++ b/test/PBL_Black_Box_Testing.xlsx
@@ -97,7 +97,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -470,13 +470,13 @@
   <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -539,12 +539,12 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Product created successfully with assigned SKU; stored in catalog with initial stock = 0 (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Product 'Apple iPad Air 11-inch' registered in MySQL database; confirmation JSON returned (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
@@ -576,12 +576,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected with validation error: 'Product ID is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Database write blocked; error response 'Product ID is required' returned (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Whitespace trimmed and rejected with error: 'Product ID is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Whitespace-only ID rejected before database execution (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Product accepted at maximum schema boundary (20 characters) and saved (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Product with 20-character SKU saved successfully in VARCHAR(20) column (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -687,12 +687,12 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected with error: 'Product name is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Missing name caught by servlet validator; emitted 'Product name is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -724,12 +724,12 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected with error: 'Category is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Empty category intercepted; returned validation error message (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -761,12 +761,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected with error: 'Unit price is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Null/empty price blocked before SQL insertion (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -798,12 +798,12 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Product accepted with minimum positive boundary price of ₹0.01 (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Minimum boundary accepted; saved with unit price ₹0.01 in DECIMAL(10,2) (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -835,12 +835,12 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected: Unit price must be strictly greater than zero (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Zero price ₹0.00 rejected with 'Unit price must be greater than zero' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -872,12 +872,12 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected: Negative pricing not allowed in warehouse catalog (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Negative value ₹-499.00 rejected with financial ledger validation error (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -909,12 +909,12 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Creation rejected: Unit price must be a valid numeric decimal (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Non-numeric string caught cleanly by NumberFormatException parser (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -946,12 +946,12 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Product accepted with high-value enterprise pricing of ₹999,999.99 (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>High-value pricing recorded without numeric overflow in database (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -983,12 +983,12 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>HTTP 409</t>
+          <t>Creation rejected with conflict error: 'Product ID already exists' (HTTP 409 Conflict)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>HTTP 409</t>
+          <t>Primary key collision intercepted; returned HTTP 409 Conflict with duplicate warning</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Description with quotes, slashes, and symbols escaped cleanly and saved (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Special characters escaped into compliant JSON without syntax crash (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -1057,12 +1057,12 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>HTML/script tags sanitized or encoded to prevent cross-site scripting (XSS) (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>HTTP 201</t>
+          <t>Input strings safely encoded; script tags neutralized upon storage (HTTP 201 Created)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1094,12 +1094,12 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Returns complete JSON array of all active warehouse inventory products (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Catalog returned with full list of electronics SKUs and stock metrics (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1131,12 +1131,12 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Returns complete product details object for specified valid Product ID (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Product record matching 'WMS-101' retrieved with all 8 attributes (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
@@ -1168,12 +1168,12 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>HTTP 404</t>
+          <t>Returns error: 'Product not found' for non-existent Product ID (HTTP 404 Not Found)</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>HTTP 404</t>
+          <t>Unknown SKU correctly mapped to standard HTTP 404 Not Found entity error</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
@@ -1205,12 +1205,12 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Product attributes (name, category, price) updated while keeping ID immutable (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Database record updated; new price and details reflected in response (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
@@ -1242,12 +1242,12 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Update rejected: Updated product name cannot be empty string (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Blank name update rejected with 'Product name is required' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
@@ -1279,12 +1279,12 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Update rejected: Updated unit price cannot be negative (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Negative price update blocked; original database value preserved (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>HTTP 404</t>
+          <t>Update rejected with 404 Not Found when target product ID does not exist (HTTP 404 Not Found)</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>HTTP 404</t>
+          <t>Non-existent SKU update intercepted; 0 rows affected mapped to HTTP 404</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
@@ -1353,12 +1353,12 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Returns live stock status table with calculated stock availability badges (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Live inventory quantities returned with In Stock / Low Stock / Out of Stock tags (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
@@ -1390,12 +1390,12 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Inward receiving adds 50 units under row-locking transaction (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Quantity incremented by +50; transaction committed atomically in MySQL (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr">
@@ -1427,12 +1427,12 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Stock quantity incremented by minimum positive integer (+1 unit) (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Smallest integer addition verified; stock increased by 1 (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
@@ -1464,12 +1464,12 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Outward dispatch decrements 20 units and confirms fulfillment (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Atomic decrement of -20 units executed under SELECT ... FOR UPDATE isolation (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G27" s="4" t="inlineStr">
@@ -1501,12 +1501,12 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Stock reduced to exactly 0 boundary; status transitions to 'Out of Stock' (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>HTTP 200</t>
+          <t>Stock depleted to 0 units cleanly without negative boundary error (HTTP 200 OK)</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1538,12 +1538,12 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Dispatch rejected: Over-reduction beyond available stock not permitted (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Transaction rolled back safely; error 'Insufficient stock available' returned (HTTP 400)</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1575,12 +1575,12 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Adjustment rejected: Quantity movement must be greater than zero (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Zero-quantity movement rejected with 'Quantity must be greater than zero' (HTTP 400)</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Adjustment rejected: Action verb must be strictly 'add' or 'reduce' (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>HTTP 400</t>
+          <t>Unsupported action 'discard' rejected with invalid action error (HTTP 400 Bad Request)</t>
         </is>
       </c>
       <c r="G31" s="4" t="inlineStr">

</xml_diff>